<commit_message>
Actualización de frecuencias y archivos del proyecto
</commit_message>
<xml_diff>
--- a/Perú V.1.xlsx
+++ b/Perú V.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CELSO HOJAS DE RUTA\FRECUENCIAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E07A5CBE-3FBD-44B6-9F93-E6E680E70EFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{895B2B52-5F89-4D93-8440-4D9DE2F5A5B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="597" xr2:uid="{461DCE75-370B-4E44-A060-84CF19771C02}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2730" uniqueCount="418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2730" uniqueCount="417">
   <si>
     <t>Country</t>
   </si>
@@ -1145,9 +1145,6 @@
     <t>VHF - AA/ALTERNA DE 119.500 MHz</t>
   </si>
   <si>
-    <t>VHF -  AA/ALTERNA DE 135.00</t>
-  </si>
-  <si>
     <t xml:space="preserve">  07° 8'35.91"S</t>
   </si>
   <si>
@@ -1229,9 +1226,6 @@
     <t xml:space="preserve"> 010°41'46.53"S</t>
   </si>
   <si>
-    <t>VHF -  AA MAIN</t>
-  </si>
-  <si>
     <t>VHF - AA/ ALTERNA DE 128.500</t>
   </si>
   <si>
@@ -1320,6 +1314,9 @@
   </si>
   <si>
     <t xml:space="preserve">AREQUIPA / SIHUAS </t>
+  </si>
+  <si>
+    <t>VHF - AA/ALTERNA DE 135.00</t>
   </si>
 </sst>
 </file>
@@ -2475,23 +2472,23 @@
         <v>42</v>
       </c>
       <c r="D2" s="42" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="E2" s="22" t="s">
         <v>235</v>
       </c>
       <c r="F2" s="46" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="G2" s="46" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="H2" s="45">
         <v>128.80000000000001</v>
       </c>
       <c r="I2" s="43"/>
       <c r="J2" s="38" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="K2" s="38"/>
       <c r="L2" s="44"/>
@@ -2515,30 +2512,30 @@
         <v>42</v>
       </c>
       <c r="D3" s="42" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="E3" s="22" t="s">
         <v>235</v>
       </c>
       <c r="F3" s="46" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="G3" s="46" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="H3" s="45">
         <v>124.75</v>
       </c>
       <c r="I3" s="43"/>
       <c r="J3" s="38" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="K3" s="38"/>
       <c r="L3" s="44"/>
       <c r="M3" s="38"/>
       <c r="N3" s="41"/>
       <c r="O3" s="41" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="P3" s="9"/>
       <c r="Q3" s="9"/>
@@ -2755,23 +2752,23 @@
         <v>42</v>
       </c>
       <c r="D9" s="29" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="E9" s="35" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="F9" s="34" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="G9" s="34" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="H9" s="21">
         <v>128.80000000000001</v>
       </c>
       <c r="I9" s="36"/>
       <c r="J9" s="39" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="K9" s="29"/>
       <c r="L9" s="30"/>
@@ -2796,30 +2793,30 @@
         <v>42</v>
       </c>
       <c r="D10" s="29" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="F10" s="34" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="G10" s="34" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="H10" s="21">
         <v>124.75</v>
       </c>
       <c r="I10" s="36"/>
       <c r="J10" s="39" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="K10" s="29"/>
       <c r="L10" s="30"/>
       <c r="M10" s="29"/>
       <c r="N10" s="20"/>
       <c r="O10" s="20" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="P10" s="20" t="s">
         <v>299</v>
@@ -2837,23 +2834,23 @@
         <v>42</v>
       </c>
       <c r="D11" s="29" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="E11" s="35" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="F11" s="34" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="G11" s="34" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="H11" s="21">
         <v>128.80000000000001</v>
       </c>
       <c r="I11" s="36"/>
       <c r="J11" s="39" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="K11" s="29"/>
       <c r="L11" s="30"/>
@@ -2878,30 +2875,30 @@
         <v>42</v>
       </c>
       <c r="D12" s="29" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="E12" s="35" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="F12" s="34" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="G12" s="34" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="H12" s="21">
         <v>124.75</v>
       </c>
       <c r="I12" s="36"/>
       <c r="J12" s="39" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="K12" s="29"/>
       <c r="L12" s="30"/>
       <c r="M12" s="29"/>
       <c r="N12" s="20"/>
       <c r="O12" s="20" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="P12" s="20" t="s">
         <v>299</v>
@@ -2925,7 +2922,7 @@
         <v>264</v>
       </c>
       <c r="F13" s="34" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="G13" s="34" t="s">
         <v>265</v>
@@ -2964,7 +2961,7 @@
         <v>264</v>
       </c>
       <c r="F14" s="34" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="G14" s="34" t="s">
         <v>265</v>
@@ -3003,7 +3000,7 @@
         <v>264</v>
       </c>
       <c r="F15" s="34" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="G15" s="34" t="s">
         <v>265</v>
@@ -3043,7 +3040,7 @@
         <v>264</v>
       </c>
       <c r="F16" s="34" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="G16" s="34" t="s">
         <v>265</v>
@@ -3083,7 +3080,7 @@
         <v>287</v>
       </c>
       <c r="F17" s="33" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="G17" s="33" t="s">
         <v>288</v>
@@ -3123,7 +3120,7 @@
         <v>287</v>
       </c>
       <c r="F18" s="33" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="G18" s="33" t="s">
         <v>288</v>
@@ -3159,23 +3156,23 @@
         <v>42</v>
       </c>
       <c r="D19" s="22" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="E19" s="26" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="F19" s="34" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="G19" s="34" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="H19" s="21">
         <v>128.5</v>
       </c>
       <c r="I19" s="36"/>
       <c r="J19" s="39" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="K19" s="29"/>
       <c r="L19" s="30"/>
@@ -3201,30 +3198,30 @@
         <v>42</v>
       </c>
       <c r="D20" s="22" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="E20" s="26" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="F20" s="34" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="G20" s="34" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="H20" s="21">
         <v>133.1</v>
       </c>
       <c r="I20" s="36"/>
       <c r="J20" s="39" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="K20" s="29"/>
       <c r="L20" s="30"/>
       <c r="M20" s="29"/>
       <c r="N20" s="29"/>
       <c r="O20" s="29" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="P20" s="20" t="s">
         <v>299</v>
@@ -3242,23 +3239,23 @@
         <v>42</v>
       </c>
       <c r="D21" s="22" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="E21" s="26" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="F21" s="34" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="G21" s="34" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="H21" s="21">
         <v>128.80000000000001</v>
       </c>
       <c r="I21" s="36"/>
       <c r="J21" s="39" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="K21" s="29"/>
       <c r="L21" s="30"/>
@@ -3283,30 +3280,30 @@
         <v>42</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="E22" s="26" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="F22" s="34" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="G22" s="34" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="H22" s="21">
         <v>124.75</v>
       </c>
       <c r="I22" s="36"/>
       <c r="J22" s="39" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="K22" s="29"/>
       <c r="L22" s="30"/>
       <c r="M22" s="29"/>
       <c r="N22" s="29"/>
       <c r="O22" s="29" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="P22" s="20" t="s">
         <v>299</v>
@@ -3330,7 +3327,7 @@
         <v>221</v>
       </c>
       <c r="F23" s="33" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="G23" s="33" t="s">
         <v>222</v>
@@ -3369,7 +3366,7 @@
         <v>221</v>
       </c>
       <c r="F24" s="33" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="G24" s="33" t="s">
         <v>222</v>
@@ -3409,7 +3406,7 @@
         <v>221</v>
       </c>
       <c r="F25" s="33" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="G25" s="33" t="s">
         <v>222</v>
@@ -3445,23 +3442,23 @@
         <v>42</v>
       </c>
       <c r="D26" s="28" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="E26" s="26" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="F26" s="34" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="G26" s="34" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="H26" s="21">
         <v>128.1</v>
       </c>
       <c r="I26" s="36"/>
       <c r="J26" s="39" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="K26" s="29"/>
       <c r="L26" s="30"/>
@@ -3486,30 +3483,30 @@
         <v>42</v>
       </c>
       <c r="D27" s="28" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="E27" s="26" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="F27" s="34" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="G27" s="34" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H27" s="21">
         <v>124.3</v>
       </c>
       <c r="I27" s="36"/>
       <c r="J27" s="39" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="K27" s="29"/>
       <c r="L27" s="30"/>
       <c r="M27" s="29"/>
       <c r="N27" s="29"/>
       <c r="O27" s="29" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="P27" s="20" t="s">
         <v>299</v>
@@ -3527,23 +3524,23 @@
         <v>42</v>
       </c>
       <c r="D28" s="28" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="E28" s="26" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="F28" s="34" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="G28" s="34" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H28" s="21">
         <v>128.5</v>
       </c>
       <c r="I28" s="36"/>
       <c r="J28" s="39" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="K28" s="29"/>
       <c r="L28" s="30"/>
@@ -3568,30 +3565,30 @@
         <v>42</v>
       </c>
       <c r="D29" s="28" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="E29" s="26" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="F29" s="34" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="G29" s="34" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H29" s="21">
         <v>133.1</v>
       </c>
       <c r="I29" s="36"/>
       <c r="J29" s="39" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="K29" s="29"/>
       <c r="L29" s="30"/>
       <c r="M29" s="29"/>
       <c r="N29" s="29"/>
       <c r="O29" s="29" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="P29" s="20" t="s">
         <v>299</v>
@@ -3977,7 +3974,7 @@
         <v>235</v>
       </c>
       <c r="F39" s="34" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="G39" s="34" t="s">
         <v>236</v>
@@ -4017,7 +4014,7 @@
         <v>235</v>
       </c>
       <c r="F40" s="34" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="G40" s="34" t="s">
         <v>236</v>
@@ -4057,7 +4054,7 @@
         <v>235</v>
       </c>
       <c r="F41" s="34" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="G41" s="34" t="s">
         <v>236</v>
@@ -4097,7 +4094,7 @@
         <v>235</v>
       </c>
       <c r="F42" s="34" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="G42" s="34" t="s">
         <v>236</v>
@@ -4137,7 +4134,7 @@
         <v>235</v>
       </c>
       <c r="F43" s="34" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="G43" s="34" t="s">
         <v>236</v>
@@ -4177,7 +4174,7 @@
         <v>235</v>
       </c>
       <c r="F44" s="34" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="G44" s="34" t="s">
         <v>236</v>
@@ -4299,7 +4296,7 @@
         <v>279</v>
       </c>
       <c r="F47" s="33" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="G47" s="33" t="s">
         <v>280</v>
@@ -4339,7 +4336,7 @@
         <v>279</v>
       </c>
       <c r="F48" s="33" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="G48" s="33" t="s">
         <v>280</v>
@@ -4539,17 +4536,17 @@
         <v>256</v>
       </c>
       <c r="F53" s="34" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="G53" s="34" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="H53" s="21">
         <v>128.5</v>
       </c>
       <c r="I53" s="36"/>
       <c r="J53" s="39" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="K53" s="29"/>
       <c r="L53" s="30"/>
@@ -4580,24 +4577,24 @@
         <v>256</v>
       </c>
       <c r="F54" s="34" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="G54" s="34" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="H54" s="21">
         <v>133.1</v>
       </c>
       <c r="I54" s="36"/>
       <c r="J54" s="39" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="K54" s="29"/>
       <c r="L54" s="30"/>
       <c r="M54" s="29"/>
       <c r="N54" s="20"/>
       <c r="O54" s="20" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="P54" s="20" t="s">
         <v>299</v>
@@ -4701,7 +4698,7 @@
         <v>293</v>
       </c>
       <c r="F57" s="33" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="G57" s="33" t="s">
         <v>294</v>
@@ -4741,7 +4738,7 @@
         <v>293</v>
       </c>
       <c r="F58" s="33" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="G58" s="33" t="s">
         <v>294</v>
@@ -4907,7 +4904,7 @@
         <v>228</v>
       </c>
       <c r="F62" s="33" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="G62" s="33" t="s">
         <v>229</v>
@@ -4947,7 +4944,7 @@
         <v>228</v>
       </c>
       <c r="F63" s="33" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="G63" s="33" t="s">
         <v>229</v>
@@ -4987,7 +4984,7 @@
         <v>228</v>
       </c>
       <c r="F64" s="33" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="G64" s="33" t="s">
         <v>229</v>
@@ -4997,7 +4994,7 @@
       </c>
       <c r="I64" s="36"/>
       <c r="J64" s="39" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="K64" s="29"/>
       <c r="L64" s="30"/>
@@ -5028,7 +5025,7 @@
         <v>228</v>
       </c>
       <c r="F65" s="33" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="G65" s="33" t="s">
         <v>229</v>
@@ -5038,14 +5035,14 @@
       </c>
       <c r="I65" s="36"/>
       <c r="J65" s="39" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="K65" s="29"/>
       <c r="L65" s="30"/>
       <c r="M65" s="29"/>
       <c r="N65" s="20"/>
       <c r="O65" s="20" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="P65" s="20" t="s">
         <v>299</v>
@@ -5069,7 +5066,7 @@
         <v>223</v>
       </c>
       <c r="F66" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G66" s="33" t="s">
         <v>224</v>
@@ -5109,7 +5106,7 @@
         <v>223</v>
       </c>
       <c r="F67" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G67" s="33" t="s">
         <v>224</v>
@@ -5149,7 +5146,7 @@
         <v>223</v>
       </c>
       <c r="F68" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G68" s="33" t="s">
         <v>224</v>
@@ -5189,7 +5186,7 @@
         <v>223</v>
       </c>
       <c r="F69" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G69" s="33" t="s">
         <v>224</v>
@@ -5229,7 +5226,7 @@
         <v>223</v>
       </c>
       <c r="F70" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G70" s="33" t="s">
         <v>224</v>
@@ -5269,7 +5266,7 @@
         <v>223</v>
       </c>
       <c r="F71" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G71" s="33" t="s">
         <v>224</v>
@@ -5309,7 +5306,7 @@
         <v>223</v>
       </c>
       <c r="F72" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G72" s="33" t="s">
         <v>224</v>
@@ -5349,7 +5346,7 @@
         <v>223</v>
       </c>
       <c r="F73" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G73" s="33" t="s">
         <v>224</v>
@@ -5389,7 +5386,7 @@
         <v>223</v>
       </c>
       <c r="F74" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G74" s="33" t="s">
         <v>224</v>
@@ -5429,7 +5426,7 @@
         <v>223</v>
       </c>
       <c r="F75" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G75" s="33" t="s">
         <v>224</v>
@@ -5469,7 +5466,7 @@
         <v>223</v>
       </c>
       <c r="F76" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G76" s="33" t="s">
         <v>224</v>
@@ -5509,7 +5506,7 @@
         <v>223</v>
       </c>
       <c r="F77" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G77" s="33" t="s">
         <v>224</v>
@@ -5549,7 +5546,7 @@
         <v>223</v>
       </c>
       <c r="F78" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G78" s="33" t="s">
         <v>224</v>
@@ -5589,7 +5586,7 @@
         <v>223</v>
       </c>
       <c r="F79" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G79" s="33" t="s">
         <v>224</v>
@@ -5629,7 +5626,7 @@
         <v>223</v>
       </c>
       <c r="F80" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G80" s="33" t="s">
         <v>224</v>
@@ -5668,7 +5665,7 @@
         <v>223</v>
       </c>
       <c r="F81" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G81" s="33" t="s">
         <v>224</v>
@@ -5707,7 +5704,7 @@
         <v>223</v>
       </c>
       <c r="F82" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G82" s="33" t="s">
         <v>224</v>
@@ -5747,7 +5744,7 @@
         <v>223</v>
       </c>
       <c r="F83" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G83" s="33" t="s">
         <v>224</v>
@@ -5787,7 +5784,7 @@
         <v>223</v>
       </c>
       <c r="F84" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G84" s="33" t="s">
         <v>224</v>
@@ -5827,7 +5824,7 @@
         <v>223</v>
       </c>
       <c r="F85" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G85" s="33" t="s">
         <v>224</v>
@@ -5866,7 +5863,7 @@
         <v>223</v>
       </c>
       <c r="F86" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G86" s="33" t="s">
         <v>224</v>
@@ -5905,7 +5902,7 @@
         <v>223</v>
       </c>
       <c r="F87" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G87" s="33" t="s">
         <v>224</v>
@@ -5945,7 +5942,7 @@
         <v>223</v>
       </c>
       <c r="F88" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G88" s="33" t="s">
         <v>224</v>
@@ -5985,7 +5982,7 @@
         <v>223</v>
       </c>
       <c r="F89" s="33" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G89" s="33" t="s">
         <v>224</v>
@@ -6025,7 +6022,7 @@
         <v>243</v>
       </c>
       <c r="F90" s="33" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="G90" s="33" t="s">
         <v>244</v>
@@ -6065,7 +6062,7 @@
         <v>243</v>
       </c>
       <c r="F91" s="33" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="G91" s="33" t="s">
         <v>244</v>
@@ -6106,7 +6103,7 @@
         <v>233</v>
       </c>
       <c r="F92" s="33" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="G92" s="33" t="s">
         <v>234</v>
@@ -6145,7 +6142,7 @@
         <v>233</v>
       </c>
       <c r="F93" s="33" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="G93" s="33" t="s">
         <v>234</v>
@@ -6185,7 +6182,7 @@
         <v>233</v>
       </c>
       <c r="F94" s="33" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="G94" s="33" t="s">
         <v>234</v>
@@ -6225,7 +6222,7 @@
         <v>233</v>
       </c>
       <c r="F95" s="33" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="G95" s="33" t="s">
         <v>234</v>
@@ -6259,30 +6256,30 @@
         <v>42</v>
       </c>
       <c r="D96" s="29" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="E96" s="26" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="F96" s="34" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="G96" s="34" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="H96" s="21">
         <v>128.5</v>
       </c>
       <c r="I96" s="36"/>
       <c r="J96" s="39" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="K96" s="29"/>
       <c r="L96" s="30"/>
       <c r="M96" s="29"/>
       <c r="N96" s="29"/>
       <c r="O96" s="29" t="s">
-        <v>387</v>
+        <v>356</v>
       </c>
       <c r="P96" s="20" t="s">
         <v>299</v>
@@ -6301,30 +6298,30 @@
         <v>42</v>
       </c>
       <c r="D97" s="29" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="E97" s="26" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="F97" s="34" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="G97" s="34" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="H97" s="21">
         <v>133.1</v>
       </c>
       <c r="I97" s="36"/>
       <c r="J97" s="39" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="K97" s="29"/>
       <c r="L97" s="30"/>
       <c r="M97" s="29"/>
       <c r="N97" s="29"/>
       <c r="O97" s="29" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="P97" s="20" t="s">
         <v>299</v>
@@ -6349,7 +6346,7 @@
         <v>245</v>
       </c>
       <c r="F98" s="33" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="G98" s="33" t="s">
         <v>246</v>
@@ -6388,7 +6385,7 @@
         <v>245</v>
       </c>
       <c r="F99" s="33" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="G99" s="33" t="s">
         <v>246</v>
@@ -6427,7 +6424,7 @@
         <v>245</v>
       </c>
       <c r="F100" s="33" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="G100" s="33" t="s">
         <v>246</v>
@@ -6467,7 +6464,7 @@
         <v>245</v>
       </c>
       <c r="F101" s="33" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="G101" s="33" t="s">
         <v>246</v>
@@ -6507,7 +6504,7 @@
         <v>245</v>
       </c>
       <c r="F102" s="33" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="G102" s="33" t="s">
         <v>246</v>
@@ -6549,7 +6546,7 @@
         <v>245</v>
       </c>
       <c r="F103" s="33" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="G103" s="33" t="s">
         <v>246</v>
@@ -6591,17 +6588,17 @@
         <v>245</v>
       </c>
       <c r="F104" s="34" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="G104" s="34" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="H104" s="21">
         <v>135</v>
       </c>
       <c r="I104" s="36"/>
       <c r="J104" s="39" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="K104" s="29"/>
       <c r="L104" s="30"/>
@@ -6633,24 +6630,24 @@
         <v>245</v>
       </c>
       <c r="F105" s="34" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="G105" s="34" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="H105" s="21">
         <v>119.1</v>
       </c>
       <c r="I105" s="36"/>
       <c r="J105" s="39" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="K105" s="29"/>
       <c r="L105" s="30"/>
       <c r="M105" s="29"/>
       <c r="N105" s="20"/>
       <c r="O105" s="20" t="s">
-        <v>359</v>
+        <v>416</v>
       </c>
       <c r="P105" s="20" t="s">
         <v>299</v>
@@ -6675,17 +6672,17 @@
         <v>245</v>
       </c>
       <c r="F106" s="34" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="G106" s="34" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="H106" s="21">
         <v>128.80000000000001</v>
       </c>
       <c r="I106" s="36"/>
       <c r="J106" s="39" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="K106" s="29"/>
       <c r="L106" s="30"/>
@@ -6716,24 +6713,24 @@
         <v>245</v>
       </c>
       <c r="F107" s="34" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="G107" s="34" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="H107" s="21">
         <v>124.75</v>
       </c>
       <c r="I107" s="36"/>
       <c r="J107" s="39" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="K107" s="29"/>
       <c r="L107" s="30"/>
       <c r="M107" s="29"/>
       <c r="N107" s="20"/>
       <c r="O107" s="20" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="P107" s="20" t="s">
         <v>299</v>
@@ -6878,17 +6875,17 @@
         <v>252</v>
       </c>
       <c r="F111" s="34" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G111" s="34" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="H111" s="21">
         <v>128.1</v>
       </c>
       <c r="I111" s="36"/>
       <c r="J111" s="20" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="K111" s="29"/>
       <c r="L111" s="30"/>
@@ -6920,24 +6917,24 @@
         <v>252</v>
       </c>
       <c r="F112" s="34" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G112" s="34" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="H112" s="21">
         <v>124.3</v>
       </c>
       <c r="I112" s="36"/>
       <c r="J112" s="20" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="K112" s="29"/>
       <c r="L112" s="30"/>
       <c r="M112" s="29"/>
       <c r="N112" s="20"/>
       <c r="O112" s="20" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="P112" s="20" t="s">
         <v>299</v>
@@ -7124,17 +7121,17 @@
         <v>215</v>
       </c>
       <c r="F117" s="34" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="G117" s="34" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="H117" s="21">
         <v>128.5</v>
       </c>
       <c r="I117" s="36"/>
       <c r="J117" s="39" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="K117" s="29"/>
       <c r="L117" s="30"/>
@@ -7165,24 +7162,24 @@
         <v>215</v>
       </c>
       <c r="F118" s="34" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="G118" s="34" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="H118" s="21">
         <v>133.1</v>
       </c>
       <c r="I118" s="36"/>
       <c r="J118" s="39" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="K118" s="29"/>
       <c r="L118" s="30"/>
       <c r="M118" s="29"/>
       <c r="N118" s="20"/>
       <c r="O118" s="20" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="P118" s="20" t="s">
         <v>299</v>
@@ -7206,7 +7203,7 @@
         <v>259</v>
       </c>
       <c r="F119" s="33" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="G119" s="33" t="s">
         <v>260</v>
@@ -7246,7 +7243,7 @@
         <v>259</v>
       </c>
       <c r="F120" s="33" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="G120" s="33" t="s">
         <v>260</v>
@@ -7286,7 +7283,7 @@
         <v>259</v>
       </c>
       <c r="F121" s="33" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="G121" s="33" t="s">
         <v>260</v>
@@ -7325,17 +7322,17 @@
         <v>259</v>
       </c>
       <c r="F122" s="34" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="G122" s="34" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="H122" s="21">
         <v>128.80000000000001</v>
       </c>
       <c r="I122" s="36"/>
       <c r="J122" s="39" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="K122" s="29"/>
       <c r="L122" s="30"/>
@@ -7366,24 +7363,24 @@
         <v>259</v>
       </c>
       <c r="F123" s="34" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="G123" s="34" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="H123" s="21">
         <v>124.75</v>
       </c>
       <c r="I123" s="36"/>
       <c r="J123" s="39" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="K123" s="29"/>
       <c r="L123" s="30"/>
       <c r="M123" s="29"/>
       <c r="N123" s="20"/>
       <c r="O123" s="20" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="P123" s="20" t="s">
         <v>299</v>
@@ -7532,7 +7529,7 @@
         <v>250</v>
       </c>
       <c r="F127" s="33" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="G127" s="33" t="s">
         <v>251</v>
@@ -7571,7 +7568,7 @@
         <v>250</v>
       </c>
       <c r="F128" s="33" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="G128" s="33" t="s">
         <v>251</v>
@@ -7610,7 +7607,7 @@
         <v>250</v>
       </c>
       <c r="F129" s="33" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="G129" s="33" t="s">
         <v>251</v>
@@ -7739,7 +7736,7 @@
       </c>
       <c r="I132" s="36"/>
       <c r="J132" s="39" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="K132" s="29"/>
       <c r="L132" s="30"/>
@@ -8174,7 +8171,7 @@
       </c>
       <c r="I143" s="36"/>
       <c r="J143" s="39" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="K143" s="29"/>
       <c r="L143" s="30"/>
@@ -8215,7 +8212,7 @@
       </c>
       <c r="I144" s="36"/>
       <c r="J144" s="39" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="K144" s="29"/>
       <c r="L144" s="30"/>
@@ -8256,7 +8253,7 @@
       </c>
       <c r="I145" s="36"/>
       <c r="J145" s="39" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="K145" s="29"/>
       <c r="L145" s="30"/>
@@ -8297,14 +8294,14 @@
       </c>
       <c r="I146" s="36"/>
       <c r="J146" s="39" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="K146" s="29"/>
       <c r="L146" s="30"/>
       <c r="M146" s="29"/>
       <c r="N146" s="29"/>
       <c r="O146" s="29" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="P146" s="20" t="s">
         <v>299</v>
@@ -8494,7 +8491,7 @@
       </c>
       <c r="I151" s="36"/>
       <c r="J151" s="39" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="K151" s="29"/>
       <c r="L151" s="30"/>
@@ -8535,14 +8532,14 @@
       </c>
       <c r="I152" s="36"/>
       <c r="J152" s="39" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="K152" s="29"/>
       <c r="L152" s="30"/>
       <c r="M152" s="29"/>
       <c r="N152" s="20"/>
       <c r="O152" s="29" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="P152" s="20" t="s">
         <v>299</v>
@@ -14155,21 +14152,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100327C040EEEBC2E4E8BDF331719AF9204" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="88684b88e321fea21b9e4a93084ec042">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9000a423-ea40-4f42-aeb8-dc93288fd0d5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a739dd0f12bf8c866a14a43425124bd7" ns2:_="">
     <xsd:import namespace="9000a423-ea40-4f42-aeb8-dc93288fd0d5"/>
@@ -14307,24 +14289,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E34F564F-6E3D-4EAB-9E28-3E787BE4233A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{36975E2A-5967-48B4-86CF-9A6B4BC252AB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3AE1F23C-6AAB-4AF9-BACE-76F8046E6C50}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -14342,6 +14322,23 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{36975E2A-5967-48B4-86CF-9A6B4BC252AB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E34F564F-6E3D-4EAB-9E28-3E787BE4233A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{e6093642-fb63-48bb-8683-d1d5da2a12ea}" enabled="0" method="" siteId="{e6093642-fb63-48bb-8683-d1d5da2a12ea}" removed="1"/>

</xml_diff>

<commit_message>
Fix: Mejorar procesamiento de coordenadas y corregir boton de reseteo de vista en el mapa
</commit_message>
<xml_diff>
--- a/Perú V.1.xlsx
+++ b/Perú V.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CELSO HOJAS DE RUTA\FRECUENCIAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{895B2B52-5F89-4D93-8440-4D9DE2F5A5B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92337CFD-1DBD-4ACD-AC92-C3D33A94BFED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="597" xr2:uid="{461DCE75-370B-4E44-A060-84CF19771C02}"/>
   </bookViews>
@@ -14152,6 +14152,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100327C040EEEBC2E4E8BDF331719AF9204" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="88684b88e321fea21b9e4a93084ec042">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9000a423-ea40-4f42-aeb8-dc93288fd0d5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a739dd0f12bf8c866a14a43425124bd7" ns2:_="">
     <xsd:import namespace="9000a423-ea40-4f42-aeb8-dc93288fd0d5"/>
@@ -14289,22 +14304,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E34F564F-6E3D-4EAB-9E28-3E787BE4233A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{36975E2A-5967-48B4-86CF-9A6B4BC252AB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3AE1F23C-6AAB-4AF9-BACE-76F8046E6C50}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -14322,23 +14339,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{36975E2A-5967-48B4-86CF-9A6B4BC252AB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E34F564F-6E3D-4EAB-9E28-3E787BE4233A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{e6093642-fb63-48bb-8683-d1d5da2a12ea}" enabled="0" method="" siteId="{e6093642-fb63-48bb-8683-d1d5da2a12ea}" removed="1"/>

</xml_diff>